<commit_message>
[feat/HD-15447] Fixed Device Calibration Report templates
</commit_message>
<xml_diff>
--- a/api/templates/device_calibration_report/fr.xlsx
+++ b/api/templates/device_calibration_report/fr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10309"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harshthakkar/Desktop/Projects/aspect/api/templates/device_calibration_report/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_calibration_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63FB4878-BCFF-C040-8395-EA40C395A5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBCEA23-AE04-7D47-BBE2-56379FE10149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="760" windowWidth="28800" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Device Calibration" sheetId="1" r:id="rId1"/>
@@ -111,12 +111,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -133,7 +131,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -152,6 +150,19 @@
         <color auto="1"/>
       </top>
       <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -176,12 +187,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -597,12 +608,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
@@ -626,13 +637,13 @@
       <c r="B8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="8" t="str">
+      <c r="E8" s="9" t="str">
         <f ca="1">IF(ISNUMBER(D8),IF(D8-TODAY()&lt;0,"OVERDUE",INT(D8-TODAY())),"")</f>
         <v/>
       </c>

</xml_diff>